<commit_message>
Update EUR->ARS rate: 2026-09-13T17:56:07Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C694"/>
+  <dimension ref="A1:C695"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12214,6 +12214,23 @@
         </is>
       </c>
     </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>17:56:06</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,846.5397</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-14T19:44:25Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C695"/>
+  <dimension ref="A1:C696"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12231,6 +12231,23 @@
         </is>
       </c>
     </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>19:44:25</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,841.5974</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-14T23:46:52Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C696"/>
+  <dimension ref="A1:C697"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12248,6 +12248,23 @@
         </is>
       </c>
     </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>23:46:52</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,841.5974</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-15T18:44:07Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C697"/>
+  <dimension ref="A1:C698"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12265,6 +12265,23 @@
         </is>
       </c>
     </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>18:44:07</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,838.9978</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-15T23:28:25Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C698"/>
+  <dimension ref="A1:C699"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12282,6 +12282,23 @@
         </is>
       </c>
     </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>23:28:25</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,838.9978</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-16T18:41:44Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C699"/>
+  <dimension ref="A1:C700"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12299,6 +12299,23 @@
         </is>
       </c>
     </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>18:41:44</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,839.3723</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-17T18:50:13Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C700"/>
+  <dimension ref="A1:C701"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12316,6 +12316,23 @@
         </is>
       </c>
     </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>18:50:13</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,827.9675</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-17T23:27:52Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C701"/>
+  <dimension ref="A1:C702"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12333,6 +12333,23 @@
         </is>
       </c>
     </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>23:27:52</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,827.9675</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-18T23:08:42Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C702"/>
+  <dimension ref="A1:C703"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12350,6 +12350,23 @@
         </is>
       </c>
     </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>23:08:42</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,830.5897</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-19T17:48:26Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C703"/>
+  <dimension ref="A1:C704"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12367,6 +12367,23 @@
         </is>
       </c>
     </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>17:48:26</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,830.5897</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-20T18:00:43Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C704"/>
+  <dimension ref="A1:C705"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12384,6 +12384,23 @@
         </is>
       </c>
     </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>18:00:43</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,830.5897</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-20T23:06:16Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C705"/>
+  <dimension ref="A1:C706"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12401,6 +12401,23 @@
         </is>
       </c>
     </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>23:06:16</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,830.5897</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-21T19:53:02Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C706"/>
+  <dimension ref="A1:C707"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12418,6 +12418,23 @@
         </is>
       </c>
     </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>19:53:02</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,829.3954</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-22T23:32:51Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C707"/>
+  <dimension ref="A1:C708"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12435,6 +12435,23 @@
         </is>
       </c>
     </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>23:32:51</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,832.0703</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-23T23:31:44Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C708"/>
+  <dimension ref="A1:C709"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12452,6 +12452,23 @@
         </is>
       </c>
     </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>23:31:44</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,824.3012</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-24T18:51:04Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C709"/>
+  <dimension ref="A1:C710"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12469,6 +12469,23 @@
         </is>
       </c>
     </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>18:51:04</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,820.0000</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-25T19:08:44Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C710"/>
+  <dimension ref="A1:C711"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12486,6 +12486,23 @@
         </is>
       </c>
     </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>19:08:44</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,829.5552</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-25T23:54:51Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C711"/>
+  <dimension ref="A1:C712"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12503,6 +12503,23 @@
         </is>
       </c>
     </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>23:54:51</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,829.5552</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-26T18:22:56Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C712"/>
+  <dimension ref="A1:C713"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12520,6 +12520,23 @@
         </is>
       </c>
     </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>18:22:56</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,829.5552</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-26T23:27:33Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C713"/>
+  <dimension ref="A1:C714"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12537,6 +12537,23 @@
         </is>
       </c>
     </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>23:27:33</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,829.5552</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-27T23:43:20Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C714"/>
+  <dimension ref="A1:C715"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12554,6 +12554,23 @@
         </is>
       </c>
     </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>23:43:20</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,829.5552</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-29T19:48:24Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C715"/>
+  <dimension ref="A1:C716"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12571,6 +12571,23 @@
         </is>
       </c>
     </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>19:48:24</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,832.6260</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-09-30T19:52:16Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C716"/>
+  <dimension ref="A1:C717"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12588,6 +12588,23 @@
         </is>
       </c>
     </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>19:52:16</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,830.5979</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-01T20:09:56Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C717"/>
+  <dimension ref="A1:C718"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12605,6 +12605,23 @@
         </is>
       </c>
     </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>20:09:56</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,815.7740</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-02T00:36:58Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C718"/>
+  <dimension ref="A1:C719"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12622,6 +12622,23 @@
         </is>
       </c>
     </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>00:36:58</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,815.7740</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-02T19:46:36Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C719"/>
+  <dimension ref="A1:C720"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12639,6 +12639,23 @@
         </is>
       </c>
     </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>19:46:36</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,821.3324</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-03T00:19:04Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C720"/>
+  <dimension ref="A1:C721"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12656,6 +12656,23 @@
         </is>
       </c>
     </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>00:19:04</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,822.3018</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-03T18:33:44Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C721"/>
+  <dimension ref="A1:C722"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12673,6 +12673,23 @@
         </is>
       </c>
     </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>18:33:44</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,822.3018</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-03T23:40:41Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C722"/>
+  <dimension ref="A1:C723"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12690,6 +12690,23 @@
         </is>
       </c>
     </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>23:40:41</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,822.3018</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-05T21:51:05Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C723"/>
+  <dimension ref="A1:C724"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12707,6 +12707,23 @@
         </is>
       </c>
     </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>21:51:04</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,802.8701</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-06T01:42:22Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C724"/>
+  <dimension ref="A1:C725"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12724,6 +12724,23 @@
         </is>
       </c>
     </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>01:42:22</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,802.8701</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-07T00:31:08Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C725"/>
+  <dimension ref="A1:C726"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12741,6 +12741,23 @@
         </is>
       </c>
     </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>00:31:08</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,805.0636</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-07T20:25:42Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C726"/>
+  <dimension ref="A1:C727"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12758,6 +12758,23 @@
         </is>
       </c>
     </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>20:25:42</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,797.5178</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-08T00:52:11Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C727"/>
+  <dimension ref="A1:C728"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12775,6 +12775,23 @@
         </is>
       </c>
     </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>00:52:10</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,797.5178</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-10T00:38:52Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C728"/>
+  <dimension ref="A1:C729"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12792,6 +12792,23 @@
         </is>
       </c>
     </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>00:38:52</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,802.5151</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-10T19:08:10Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C729"/>
+  <dimension ref="A1:C730"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12809,6 +12809,23 @@
         </is>
       </c>
     </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>19:08:10</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,802.5151</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-11T00:10:27Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C730"/>
+  <dimension ref="A1:C731"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12826,6 +12826,23 @@
         </is>
       </c>
     </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>00:10:27</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,802.5151</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-11T19:22:10Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C731"/>
+  <dimension ref="A1:C732"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12843,6 +12843,23 @@
         </is>
       </c>
     </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>19:22:10</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,802.5151</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-12T00:22:14Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C732"/>
+  <dimension ref="A1:C733"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12860,6 +12860,23 @@
         </is>
       </c>
     </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>00:22:14</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,802.5151</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-12T22:24:14Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C733"/>
+  <dimension ref="A1:C734"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12877,6 +12877,23 @@
         </is>
       </c>
     </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>22:24:13</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,799.1838</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-13T20:31:15Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C734"/>
+  <dimension ref="A1:C735"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12894,6 +12894,23 @@
         </is>
       </c>
     </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>20:31:15</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,799.0229</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-14T00:12:30Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C735"/>
+  <dimension ref="A1:C736"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12911,6 +12911,23 @@
         </is>
       </c>
     </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>00:12:30</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,799.0229</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-14T23:47:50Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C736"/>
+  <dimension ref="A1:C737"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12928,6 +12928,23 @@
         </is>
       </c>
     </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>23:47:49</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,803.0312</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-15T18:53:45Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C737"/>
+  <dimension ref="A1:C738"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12945,6 +12945,23 @@
         </is>
       </c>
     </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>18:53:45</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,811.6644</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-16T18:38:27Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C738"/>
+  <dimension ref="A1:C739"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12962,6 +12962,23 @@
         </is>
       </c>
     </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>18:38:27</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,818.8080</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-17T17:46:27Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C739"/>
+  <dimension ref="A1:C740"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12979,6 +12979,23 @@
         </is>
       </c>
     </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>17:46:27</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,815.8424</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-17T22:58:45Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C740"/>
+  <dimension ref="A1:C741"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12996,6 +12996,23 @@
         </is>
       </c>
     </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>22:58:45</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,815.8424</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-19T20:23:33Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C741"/>
+  <dimension ref="A1:C742"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13013,6 +13013,23 @@
         </is>
       </c>
     </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>20:23:33</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,814.4569</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-20T00:10:43Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C742"/>
+  <dimension ref="A1:C743"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13030,6 +13030,23 @@
         </is>
       </c>
     </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>00:10:43</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,814.4569</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-20T23:42:29Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C743"/>
+  <dimension ref="A1:C744"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13047,6 +13047,23 @@
         </is>
       </c>
     </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>23:42:29</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,820.6814</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-21T19:07:48Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C744"/>
+  <dimension ref="A1:C745"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13064,6 +13064,23 @@
         </is>
       </c>
     </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>19:07:47</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,826.6160</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-21T23:56:46Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C745"/>
+  <dimension ref="A1:C746"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13081,6 +13081,23 @@
         </is>
       </c>
     </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>23:56:46</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,826.6160</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-22T19:03:49Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C746"/>
+  <dimension ref="A1:C747"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13098,6 +13098,23 @@
         </is>
       </c>
     </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>19:03:49</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,829.6558</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-22T23:56:05Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C747"/>
+  <dimension ref="A1:C748"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13115,6 +13115,23 @@
         </is>
       </c>
     </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>23:56:05</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,829.6558</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-23T23:47:53Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C748"/>
+  <dimension ref="A1:C749"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13132,6 +13132,23 @@
         </is>
       </c>
     </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>23:47:53</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,840.7049</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-24T23:02:08Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C749"/>
+  <dimension ref="A1:C750"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13149,6 +13149,23 @@
         </is>
       </c>
     </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>23:02:08</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,840.7049</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-25T18:10:59Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C750"/>
+  <dimension ref="A1:C751"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13166,6 +13166,23 @@
         </is>
       </c>
     </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>18:10:59</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,840.7049</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-27T00:17:48Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C751"/>
+  <dimension ref="A1:C752"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13183,6 +13183,23 @@
         </is>
       </c>
     </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>00:17:48</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,842.6623</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-28T20:05:23Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C752"/>
+  <dimension ref="A1:C753"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13200,6 +13200,23 @@
         </is>
       </c>
     </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>20:05:23</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,843.9688</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-29T00:41:38Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C753"/>
+  <dimension ref="A1:C754"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13217,6 +13217,23 @@
         </is>
       </c>
     </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>00:41:38</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,843.9688</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-29T20:04:49Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C754"/>
+  <dimension ref="A1:C755"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13234,6 +13234,23 @@
         </is>
       </c>
     </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>20:04:49</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,841.8944</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-30T00:42:03Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C755"/>
+  <dimension ref="A1:C756"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13251,6 +13251,23 @@
         </is>
       </c>
     </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>00:42:03</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,841.8944</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update EUR->ARS rate: 2026-10-31T00:35:07Z
</commit_message>
<xml_diff>
--- a/wu_eur_ars.xlsx
+++ b/wu_eur_ars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C756"/>
+  <dimension ref="A1:C757"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13268,6 +13268,23 @@
         </is>
       </c>
     </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>00:35:07</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>1.00 EUR = 1,846.8260</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>